<commit_message>
changes adding global south
</commit_message>
<xml_diff>
--- a/tools_register.xlsx
+++ b/tools_register.xlsx
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J16"/>
+  <dimension ref="A1:J33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -1255,6 +1255,798 @@
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>RECreation (INESC TEC)</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>INESC TEC (Portugal)</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Platform to size and manage renewable energy communities and collective self-consumption</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>Modular; dynamic allocation coefficients and compensation flows between members</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>Smart-meter data (via the grid operator)</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>Allocation coefficients, self-consumption, compensation flows</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>Licensed (per public description)</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>https://www.inesctec.pt/en</t>
+        </is>
+      </c>
+      <c r="J17" s="2" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>E-REDES Collective Self-consumption Manager (Portugal)</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>E-REDES, distribution system operator (Portugal)</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Grid-operator portal for collective self-consumption and energy communities</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>Sharing coefficients applied by the operator: fixed, proportional, hierarchical or dynamic</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>Operator's own metering data</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>Sharing coefficients per member and period</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>Operator service</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>https://www.e-redes.pt/en/sharing-coefficients</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>EnergyID (Belgium, Netherlands)</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>EnergyID (Belgium)</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Member dashboards and scorecards; simulator for new participants</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>Collective self-consumption analysis from smart-meter data</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>Smart-meter and device data, member consent</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>Self-consumption and sharing per member</t>
+        </is>
+      </c>
+      <c r="H19" s="3" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I19" s="2" t="inlineStr">
+        <is>
+          <t>https://www.energyid.eu/en/solutions/energy-communities/</t>
+        </is>
+      </c>
+      <c r="J19" s="2" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>Communit-e (CIRCE)</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>CIRCE Technology Centre (Spain)</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>Community management portal</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>User management and personalised distribution coefficients</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>Smart-meter data</t>
+        </is>
+      </c>
+      <c r="G20" s="3" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="H20" s="3" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t>https://www.fcirce.es</t>
+        </is>
+      </c>
+      <c r="J20" s="2" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>OYO Communities (France)</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>Company (France)</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>Allocation keys for collective self-consumption; approved by the grid operator Enedis (per vendor)</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>Operator metering data</t>
+        </is>
+      </c>
+      <c r="G21" s="3" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>Proprietary</t>
+        </is>
+      </c>
+      <c r="I21" s="2" t="n"/>
+      <c r="J21" s="2" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>Austrian energy-sharing data stack (EDA market communication, EDDIE, ISEG interface)</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Grid operators, market operators, Horizon Europe project EDDIE</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>Standard market-communication platform with the smart meter as the data source; EDDIE open-source data-access framework; interoperable interface initiative (ISEG)</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>Standardised market messages (details to check)</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>Smart-meter data under consent</t>
+        </is>
+      </c>
+      <c r="G22" s="3" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>EDDIE open source (Apache 2.0)</t>
+        </is>
+      </c>
+      <c r="I22" s="2" t="n"/>
+      <c r="J22" s="2" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>Energy Local Club (UK)</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>Energy Local (UK community interest company)</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>Club statements for members</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>Half-hourly matching of local generation and member demand, with a 'match' tariff through one supplier</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>Half-hourly smart-meter data</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>Share of demand matched with local generation (52% reported in the first Bethesda club, about 2018)</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>Open model, supplier partnership</t>
+        </is>
+      </c>
+      <c r="I23" s="2" t="inlineStr">
+        <is>
+          <t>https://ashden.org/winners/energy-local</t>
+        </is>
+      </c>
+      <c r="J23" s="2" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>Peer-to-peer trading platforms (Brooklyn Microgrid / LO3, Power Ledger, Vandebron)</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>Companies (US, Australia, Netherlands)</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>Trading apps</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>Local markets, often blockchain-based</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>Smart-meter data</t>
+        </is>
+      </c>
+      <c r="G24" s="3" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>Proprietary</t>
+        </is>
+      </c>
+      <c r="I24" s="2" t="inlineStr">
+        <is>
+          <t>https://microgridknowledge.com/community-microgrid-brooklyn/</t>
+        </is>
+      </c>
+      <c r="J24" s="2" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>Virtual and community net metering in Canada (Ontario demonstration, SolarShare, City of Nelson)</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>Ontario regulation O. Reg. 679/21 and local projects</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>Utility billing credits allocated to participants (rules, not a software tool)</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>Utility meter data</t>
+        </is>
+      </c>
+      <c r="G25" s="3" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>Regulatory scheme</t>
+        </is>
+      </c>
+      <c r="I25" s="2" t="n"/>
+      <c r="J25" s="2" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>FlexMeasures (Seita; LF Energy)</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>Seita, LF Energy incubation (Netherlands)</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>Dashboard and API</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>Open-source energy management: schedules batteries, heat pumps and V2G; asset grouping</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>Sensors and assets (details to check)</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>Time-series from meters and devices</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>Costs, peak and self-consumption outcomes of schedules</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>Open source (Apache 2.0)</t>
+        </is>
+      </c>
+      <c r="I26" s="2" t="inlineStr">
+        <is>
+          <t>https://flexmeasures.io</t>
+        </is>
+      </c>
+      <c r="J26" s="2" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>OpenEMS (open-source energy management system)</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>OpenEMS community</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>Web UI</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>Java open-source EMS for storage and PV; peak shaving and self-consumption control</t>
+        </is>
+      </c>
+      <c r="E27" s="3" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>Device protocols (Modbus and others)</t>
+        </is>
+      </c>
+      <c r="G27" s="3" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="H27" s="2" t="inlineStr">
+        <is>
+          <t>Open source</t>
+        </is>
+      </c>
+      <c r="I27" s="2" t="inlineStr">
+        <is>
+          <t>https://openems.io</t>
+        </is>
+      </c>
+      <c r="J27" s="2" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>Piclo Flex (flexibility marketplace)</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>Piclo (UK)</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>Marketplace for flexibility providers and grid operators</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>Competitions run by distribution grid operators; used in several countries</t>
+        </is>
+      </c>
+      <c r="E28" s="3" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>Asset registration and dispatch data</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>Claims over 3 GW of flexibility contracts enabled (June 2025, vendor figure, unverified)</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>Proprietary</t>
+        </is>
+      </c>
+      <c r="I28" s="2" t="inlineStr">
+        <is>
+          <t>https://piclo.energy/flex</t>
+        </is>
+      </c>
+      <c r="J28" s="2" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>EU flexibility projects for communities (FLEXCoop, DEDALUS, Scaling-up Power Flexible Communities)</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>Horizon 2020 and Horizon Europe consortia</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>Aggregator and consumer interfaces</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>Flexibility forecasting, aggregation and measurement and verification of consumer response</t>
+        </is>
+      </c>
+      <c r="E29" s="3" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>Smart-meter and device data</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>Peak reduction and system cost targets (DEDALUS aims at 15%)</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="I29" s="2" t="n"/>
+      <c r="J29" s="2" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>Project LEO, Local Energy Oxfordshire (2019 to 2023)</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>SSEN, Oxford, Low Carbon Hub and partners (UK)</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>Resident engagement; trading and market platforms</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>Distribution-grid flexibility market trials, peer-to-peer network capacity trading, local area energy planning</t>
+        </is>
+      </c>
+      <c r="E30" s="3" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>More than 100 monitoring stations</t>
+        </is>
+      </c>
+      <c r="G30" s="3" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
+          <t>Final report public</t>
+        </is>
+      </c>
+      <c r="I30" s="2" t="inlineStr">
+        <is>
+          <t>https://www.lowcarbonhub.org/wp-content/uploads/2023/02/LEO-Final-Report-Web_lr.pdf</t>
+        </is>
+      </c>
+      <c r="J30" s="2" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>Energy community KPI framework (Giannuzzo et al., Energy Reports 2025)</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>Academic paper (Italy)</t>
+        </is>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>Framework, not software</t>
+        </is>
+      </c>
+      <c r="E31" s="3" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="F31" s="3" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="inlineStr">
+        <is>
+          <t>25 KPIs in four domains: energy, economic, social, environmental; for planning, operation, monitoring and benchmarking</t>
+        </is>
+      </c>
+      <c r="H31" s="2" t="inlineStr">
+        <is>
+          <t>Paper</t>
+        </is>
+      </c>
+      <c r="I31" s="2" t="n"/>
+      <c r="J31" s="2" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>Integrated Energy Community Performance Index (IECPI)</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>Academic proposal</t>
+        </is>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>Composite index, not software</t>
+        </is>
+      </c>
+      <c r="E32" s="3" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="F32" s="3" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>Composite performance index (components to check)</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="inlineStr">
+        <is>
+          <t>Paper</t>
+        </is>
+      </c>
+      <c r="I32" s="2" t="n"/>
+      <c r="J32" s="2" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>Smart Energy Communities Benchmark (QUEST and Pollution Probe, 2020)</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>QUEST Canada and Pollution Probe</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>Assessment per municipality</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>Self-assessment against ten indicators</t>
+        </is>
+      </c>
+      <c r="E33" s="3" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>Municipal self-reporting; nine pilot communities</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="inlineStr">
+        <is>
+          <t>Ten indicators: five on capacity (governance, staff, data, financials, strategy), five on outcomes (land use, energy networks, water and waste, transportation, buildings)</t>
+        </is>
+      </c>
+      <c r="H33" s="2" t="inlineStr">
+        <is>
+          <t>Public report</t>
+        </is>
+      </c>
+      <c r="I33" s="2" t="inlineStr">
+        <is>
+          <t>https://questcanada.org/project/is-your-community-energy-smart/</t>
+        </is>
+      </c>
+      <c r="J33" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
changes adding global south and azimut
</commit_message>
<xml_diff>
--- a/tools_register.xlsx
+++ b/tools_register.xlsx
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J33"/>
+  <dimension ref="A1:J36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -1259,22 +1259,22 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>RECreation (INESC TEC)</t>
+          <t>OnSSET, Open Source Spatial Electrification Toolkit (KTH)</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>INESC TEC (Portugal)</t>
-        </is>
-      </c>
-      <c r="C17" s="2" t="inlineStr">
-        <is>
-          <t>Platform to size and manage renewable energy communities and collective self-consumption</t>
+          <t>KTH dESA, Sweden</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>?</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>Modular; dynamic allocation coefficients and compensation flows between members</t>
+          <t>GIS-based least-cost comparison of grid extension, mini-grids and stand-alone systems</t>
         </is>
       </c>
       <c r="E17" s="3" t="inlineStr">
@@ -1284,22 +1284,22 @@
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>Smart-meter data (via the grid operator)</t>
+          <t>Spatial datasets (population, grid, resources)</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>Allocation coefficients, self-consumption, compensation flows</t>
+          <t>Least-cost electrification option and cost per location</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>Licensed (per public description)</t>
+          <t>Open source</t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>https://www.inesctec.pt/en</t>
+          <t>https://onsset.readthedocs.io/</t>
         </is>
       </c>
       <c r="J17" s="2" t="inlineStr"/>
@@ -1307,22 +1307,22 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>E-REDES Collective Self-consumption Manager (Portugal)</t>
+          <t>OnSSET for Mini Grids (OMG)</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>E-REDES, distribution system operator (Portugal)</t>
-        </is>
-      </c>
-      <c r="C18" s="2" t="inlineStr">
-        <is>
-          <t>Grid-operator portal for collective self-consumption and energy communities</t>
+          <t>OnSSET community</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>?</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>Sharing coefficients applied by the operator: fixed, proportional, hierarchical or dynamic</t>
+          <t>Python tool: hybrid solar-diesel-storage sizing and distribution design with bill of quantities; stand-alone or inside a national least-cost model</t>
         </is>
       </c>
       <c r="E18" s="3" t="inlineStr">
@@ -1332,22 +1332,22 @@
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>Operator's own metering data</t>
+          <t>Site and spatial data</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>Sharing coefficients per member and period</t>
+          <t>Levelised cost of electricity, bill of quantities</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>Operator service</t>
+          <t>Open source</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>https://www.e-redes.pt/en/sharing-coefficients</t>
+          <t>https://omg-userguide.readthedocs.io</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr"/>
@@ -1355,22 +1355,22 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>EnergyID (Belgium, Netherlands)</t>
+          <t>MicroGridsPy</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>EnergyID (Belgium)</t>
-        </is>
-      </c>
-      <c r="C19" s="2" t="inlineStr">
-        <is>
-          <t>Member dashboards and scorecards; simulator for new participants</t>
+          <t>Research groups (to confirm)</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>?</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>Collective self-consumption analysis from smart-meter data</t>
+          <t>Optimisation of microgrid sizing; a 2026 master's thesis found OnSSET overestimates mini-grid costs against it on Kenyan sites (preliminary)</t>
         </is>
       </c>
       <c r="E19" s="3" t="inlineStr">
@@ -1378,14 +1378,14 @@
           <t>?</t>
         </is>
       </c>
-      <c r="F19" s="2" t="inlineStr">
-        <is>
-          <t>Smart-meter and device data, member consent</t>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>?</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>Self-consumption and sharing per member</t>
+          <t>Levelised cost of electricity</t>
         </is>
       </c>
       <c r="H19" s="3" t="inlineStr">
@@ -1393,32 +1393,28 @@
           <t>?</t>
         </is>
       </c>
-      <c r="I19" s="2" t="inlineStr">
-        <is>
-          <t>https://www.energyid.eu/en/solutions/energy-communities/</t>
-        </is>
-      </c>
+      <c r="I19" s="2" t="n"/>
       <c r="J19" s="2" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Communit-e (CIRCE)</t>
+          <t>RECreation (INESC TEC)</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>CIRCE Technology Centre (Spain)</t>
+          <t>INESC TEC (Portugal)</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Community management portal</t>
+          <t>Platform to size and manage renewable energy communities and collective self-consumption</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>User management and personalised distribution coefficients</t>
+          <t>Modular; dynamic allocation coefficients and compensation flows between members</t>
         </is>
       </c>
       <c r="E20" s="3" t="inlineStr">
@@ -1428,22 +1424,22 @@
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>Smart-meter data</t>
-        </is>
-      </c>
-      <c r="G20" s="3" t="inlineStr">
-        <is>
-          <t>?</t>
-        </is>
-      </c>
-      <c r="H20" s="3" t="inlineStr">
-        <is>
-          <t>?</t>
+          <t>Smart-meter data (via the grid operator)</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>Allocation coefficients, self-consumption, compensation flows</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>Licensed (per public description)</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>https://www.fcirce.es</t>
+          <t>https://www.inesctec.pt/en</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr"/>
@@ -1451,22 +1447,22 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>OYO Communities (France)</t>
+          <t>E-REDES Collective Self-consumption Manager (Portugal)</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Company (France)</t>
-        </is>
-      </c>
-      <c r="C21" s="3" t="inlineStr">
-        <is>
-          <t>?</t>
+          <t>E-REDES, distribution system operator (Portugal)</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>Grid-operator portal for collective self-consumption and energy communities</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>Allocation keys for collective self-consumption; approved by the grid operator Enedis (per vendor)</t>
+          <t>Sharing coefficients applied by the operator: fixed, proportional, hierarchical or dynamic</t>
         </is>
       </c>
       <c r="E21" s="3" t="inlineStr">
@@ -1476,85 +1472,93 @@
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>Operator metering data</t>
-        </is>
-      </c>
-      <c r="G21" s="3" t="inlineStr">
-        <is>
-          <t>?</t>
+          <t>Operator's own metering data</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>Sharing coefficients per member and period</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>Proprietary</t>
-        </is>
-      </c>
-      <c r="I21" s="2" t="n"/>
+          <t>Operator service</t>
+        </is>
+      </c>
+      <c r="I21" s="2" t="inlineStr">
+        <is>
+          <t>https://www.e-redes.pt/en/sharing-coefficients</t>
+        </is>
+      </c>
       <c r="J21" s="2" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Austrian energy-sharing data stack (EDA market communication, EDDIE, ISEG interface)</t>
+          <t>EnergyID (Belgium, Netherlands)</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Grid operators, market operators, Horizon Europe project EDDIE</t>
-        </is>
-      </c>
-      <c r="C22" s="3" t="inlineStr">
-        <is>
-          <t>?</t>
+          <t>EnergyID (Belgium)</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>Member dashboards and scorecards; simulator for new participants</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>Standard market-communication platform with the smart meter as the data source; EDDIE open-source data-access framework; interoperable interface initiative (ISEG)</t>
-        </is>
-      </c>
-      <c r="E22" s="2" t="inlineStr">
-        <is>
-          <t>Standardised market messages (details to check)</t>
+          <t>Collective self-consumption analysis from smart-meter data</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>?</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>Smart-meter data under consent</t>
-        </is>
-      </c>
-      <c r="G22" s="3" t="inlineStr">
-        <is>
-          <t>?</t>
-        </is>
-      </c>
-      <c r="H22" s="2" t="inlineStr">
-        <is>
-          <t>EDDIE open source (Apache 2.0)</t>
-        </is>
-      </c>
-      <c r="I22" s="2" t="n"/>
+          <t>Smart-meter and device data, member consent</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>Self-consumption and sharing per member</t>
+        </is>
+      </c>
+      <c r="H22" s="3" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>https://www.energyid.eu/en/solutions/energy-communities/</t>
+        </is>
+      </c>
       <c r="J22" s="2" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>Energy Local Club (UK)</t>
+          <t>Communit-e (CIRCE)</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Energy Local (UK community interest company)</t>
+          <t>CIRCE Technology Centre (Spain)</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Club statements for members</t>
+          <t>Community management portal</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>Half-hourly matching of local generation and member demand, with a 'match' tariff through one supplier</t>
+          <t>User management and personalised distribution coefficients</t>
         </is>
       </c>
       <c r="E23" s="3" t="inlineStr">
@@ -1564,22 +1568,22 @@
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>Half-hourly smart-meter data</t>
-        </is>
-      </c>
-      <c r="G23" s="2" t="inlineStr">
-        <is>
-          <t>Share of demand matched with local generation (52% reported in the first Bethesda club, about 2018)</t>
-        </is>
-      </c>
-      <c r="H23" s="2" t="inlineStr">
-        <is>
-          <t>Open model, supplier partnership</t>
+          <t>Smart-meter data</t>
+        </is>
+      </c>
+      <c r="G23" s="3" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="H23" s="3" t="inlineStr">
+        <is>
+          <t>?</t>
         </is>
       </c>
       <c r="I23" s="2" t="inlineStr">
         <is>
-          <t>https://ashden.org/winners/energy-local</t>
+          <t>https://www.fcirce.es</t>
         </is>
       </c>
       <c r="J23" s="2" t="inlineStr"/>
@@ -1587,22 +1591,22 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Peer-to-peer trading platforms (Brooklyn Microgrid / LO3, Power Ledger, Vandebron)</t>
+          <t>OYO Communities (France)</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>Companies (US, Australia, Netherlands)</t>
-        </is>
-      </c>
-      <c r="C24" s="2" t="inlineStr">
-        <is>
-          <t>Trading apps</t>
+          <t>Company (France)</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>?</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>Local markets, often blockchain-based</t>
+          <t>Allocation keys for collective self-consumption; approved by the grid operator Enedis (per vendor)</t>
         </is>
       </c>
       <c r="E24" s="3" t="inlineStr">
@@ -1612,7 +1616,7 @@
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>Smart-meter data</t>
+          <t>Operator metering data</t>
         </is>
       </c>
       <c r="G24" s="3" t="inlineStr">
@@ -1625,22 +1629,18 @@
           <t>Proprietary</t>
         </is>
       </c>
-      <c r="I24" s="2" t="inlineStr">
-        <is>
-          <t>https://microgridknowledge.com/community-microgrid-brooklyn/</t>
-        </is>
-      </c>
+      <c r="I24" s="2" t="n"/>
       <c r="J24" s="2" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>Virtual and community net metering in Canada (Ontario demonstration, SolarShare, City of Nelson)</t>
+          <t>Austrian energy-sharing data stack (EDA market communication, EDDIE, ISEG interface)</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Ontario regulation O. Reg. 679/21 and local projects</t>
+          <t>Grid operators, market operators, Horizon Europe project EDDIE</t>
         </is>
       </c>
       <c r="C25" s="3" t="inlineStr">
@@ -1650,17 +1650,17 @@
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>Utility billing credits allocated to participants (rules, not a software tool)</t>
-        </is>
-      </c>
-      <c r="E25" s="3" t="inlineStr">
-        <is>
-          <t>?</t>
+          <t>Standard market-communication platform with the smart meter as the data source; EDDIE open-source data-access framework; interoperable interface initiative (ISEG)</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>Standardised market messages (details to check)</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>Utility meter data</t>
+          <t>Smart-meter data under consent</t>
         </is>
       </c>
       <c r="G25" s="3" t="inlineStr">
@@ -1670,7 +1670,7 @@
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>Regulatory scheme</t>
+          <t>EDDIE open source (Apache 2.0)</t>
         </is>
       </c>
       <c r="I25" s="2" t="n"/>
@@ -1679,47 +1679,47 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>FlexMeasures (Seita; LF Energy)</t>
+          <t>Energy Local Club (UK)</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Seita, LF Energy incubation (Netherlands)</t>
+          <t>Energy Local (UK community interest company)</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Dashboard and API</t>
+          <t>Club statements for members</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>Open-source energy management: schedules batteries, heat pumps and V2G; asset grouping</t>
-        </is>
-      </c>
-      <c r="E26" s="2" t="inlineStr">
-        <is>
-          <t>Sensors and assets (details to check)</t>
+          <t>Half-hourly matching of local generation and member demand, with a 'match' tariff through one supplier</t>
+        </is>
+      </c>
+      <c r="E26" s="3" t="inlineStr">
+        <is>
+          <t>?</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>Time-series from meters and devices</t>
+          <t>Half-hourly smart-meter data</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>Costs, peak and self-consumption outcomes of schedules</t>
+          <t>Share of demand matched with local generation (52% reported in the first Bethesda club, about 2018)</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>Open source (Apache 2.0)</t>
+          <t>Open model, supplier partnership</t>
         </is>
       </c>
       <c r="I26" s="2" t="inlineStr">
         <is>
-          <t>https://flexmeasures.io</t>
+          <t>https://ashden.org/winners/energy-local</t>
         </is>
       </c>
       <c r="J26" s="2" t="inlineStr"/>
@@ -1727,22 +1727,22 @@
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>OpenEMS (open-source energy management system)</t>
+          <t>Peer-to-peer trading platforms (Brooklyn Microgrid / LO3, Power Ledger, Vandebron)</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>OpenEMS community</t>
+          <t>Companies (US, Australia, Netherlands)</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Web UI</t>
+          <t>Trading apps</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>Java open-source EMS for storage and PV; peak shaving and self-consumption control</t>
+          <t>Local markets, often blockchain-based</t>
         </is>
       </c>
       <c r="E27" s="3" t="inlineStr">
@@ -1752,7 +1752,7 @@
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>Device protocols (Modbus and others)</t>
+          <t>Smart-meter data</t>
         </is>
       </c>
       <c r="G27" s="3" t="inlineStr">
@@ -1762,12 +1762,12 @@
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
-          <t>Open source</t>
+          <t>Proprietary</t>
         </is>
       </c>
       <c r="I27" s="2" t="inlineStr">
         <is>
-          <t>https://openems.io</t>
+          <t>https://microgridknowledge.com/community-microgrid-brooklyn/</t>
         </is>
       </c>
       <c r="J27" s="2" t="inlineStr"/>
@@ -1775,22 +1775,22 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Piclo Flex (flexibility marketplace)</t>
+          <t>Virtual and community net metering in Canada (Ontario demonstration, SolarShare, City of Nelson)</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Piclo (UK)</t>
-        </is>
-      </c>
-      <c r="C28" s="2" t="inlineStr">
-        <is>
-          <t>Marketplace for flexibility providers and grid operators</t>
+          <t>Ontario regulation O. Reg. 679/21 and local projects</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>?</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>Competitions run by distribution grid operators; used in several countries</t>
+          <t>Utility billing credits allocated to participants (rules, not a software tool)</t>
         </is>
       </c>
       <c r="E28" s="3" t="inlineStr">
@@ -1800,89 +1800,89 @@
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>Asset registration and dispatch data</t>
-        </is>
-      </c>
-      <c r="G28" s="2" t="inlineStr">
-        <is>
-          <t>Claims over 3 GW of flexibility contracts enabled (June 2025, vendor figure, unverified)</t>
+          <t>Utility meter data</t>
+        </is>
+      </c>
+      <c r="G28" s="3" t="inlineStr">
+        <is>
+          <t>?</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>Proprietary</t>
-        </is>
-      </c>
-      <c r="I28" s="2" t="inlineStr">
-        <is>
-          <t>https://piclo.energy/flex</t>
-        </is>
-      </c>
+          <t>Regulatory scheme</t>
+        </is>
+      </c>
+      <c r="I28" s="2" t="n"/>
       <c r="J28" s="2" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>EU flexibility projects for communities (FLEXCoop, DEDALUS, Scaling-up Power Flexible Communities)</t>
+          <t>FlexMeasures (Seita; LF Energy)</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>Horizon 2020 and Horizon Europe consortia</t>
+          <t>Seita, LF Energy incubation (Netherlands)</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Aggregator and consumer interfaces</t>
+          <t>Dashboard and API</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>Flexibility forecasting, aggregation and measurement and verification of consumer response</t>
-        </is>
-      </c>
-      <c r="E29" s="3" t="inlineStr">
-        <is>
-          <t>?</t>
+          <t>Open-source energy management: schedules batteries, heat pumps and V2G; asset grouping</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>Sensors and assets (details to check)</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>Smart-meter and device data</t>
+          <t>Time-series from meters and devices</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>Peak reduction and system cost targets (DEDALUS aims at 15%)</t>
+          <t>Costs, peak and self-consumption outcomes of schedules</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>Mixed</t>
-        </is>
-      </c>
-      <c r="I29" s="2" t="n"/>
+          <t>Open source (Apache 2.0)</t>
+        </is>
+      </c>
+      <c r="I29" s="2" t="inlineStr">
+        <is>
+          <t>https://flexmeasures.io</t>
+        </is>
+      </c>
       <c r="J29" s="2" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Project LEO, Local Energy Oxfordshire (2019 to 2023)</t>
+          <t>OpenEMS (open-source energy management system)</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>SSEN, Oxford, Low Carbon Hub and partners (UK)</t>
+          <t>OpenEMS community</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Resident engagement; trading and market platforms</t>
+          <t>Web UI</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>Distribution-grid flexibility market trials, peer-to-peer network capacity trading, local area energy planning</t>
+          <t>Java open-source EMS for storage and PV; peak shaving and self-consumption control</t>
         </is>
       </c>
       <c r="E30" s="3" t="inlineStr">
@@ -1892,7 +1892,7 @@
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>More than 100 monitoring stations</t>
+          <t>Device protocols (Modbus and others)</t>
         </is>
       </c>
       <c r="G30" s="3" t="inlineStr">
@@ -1902,12 +1902,12 @@
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>Final report public</t>
+          <t>Open source</t>
         </is>
       </c>
       <c r="I30" s="2" t="inlineStr">
         <is>
-          <t>https://www.lowcarbonhub.org/wp-content/uploads/2023/02/LEO-Final-Report-Web_lr.pdf</t>
+          <t>https://openems.io</t>
         </is>
       </c>
       <c r="J30" s="2" t="inlineStr"/>
@@ -1915,22 +1915,22 @@
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>Energy community KPI framework (Giannuzzo et al., Energy Reports 2025)</t>
+          <t>Piclo Flex (flexibility marketplace)</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>Academic paper (Italy)</t>
-        </is>
-      </c>
-      <c r="C31" s="3" t="inlineStr">
-        <is>
-          <t>?</t>
+          <t>Piclo (UK)</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>Marketplace for flexibility providers and grid operators</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>Framework, not software</t>
+          <t>Competitions run by distribution grid operators; used in several countries</t>
         </is>
       </c>
       <c r="E31" s="3" t="inlineStr">
@@ -1938,43 +1938,47 @@
           <t>?</t>
         </is>
       </c>
-      <c r="F31" s="3" t="inlineStr">
-        <is>
-          <t>?</t>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>Asset registration and dispatch data</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>25 KPIs in four domains: energy, economic, social, environmental; for planning, operation, monitoring and benchmarking</t>
+          <t>Claims over 3 GW of flexibility contracts enabled (June 2025, vendor figure, unverified)</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
-          <t>Paper</t>
-        </is>
-      </c>
-      <c r="I31" s="2" t="n"/>
+          <t>Proprietary</t>
+        </is>
+      </c>
+      <c r="I31" s="2" t="inlineStr">
+        <is>
+          <t>https://piclo.energy/flex</t>
+        </is>
+      </c>
       <c r="J31" s="2" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>Integrated Energy Community Performance Index (IECPI)</t>
+          <t>EU flexibility projects for communities (FLEXCoop, DEDALUS, Scaling-up Power Flexible Communities)</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>Academic proposal</t>
-        </is>
-      </c>
-      <c r="C32" s="3" t="inlineStr">
-        <is>
-          <t>?</t>
+          <t>Horizon 2020 and Horizon Europe consortia</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>Aggregator and consumer interfaces</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>Composite index, not software</t>
+          <t>Flexibility forecasting, aggregation and measurement and verification of consumer response</t>
         </is>
       </c>
       <c r="E32" s="3" t="inlineStr">
@@ -1982,19 +1986,19 @@
           <t>?</t>
         </is>
       </c>
-      <c r="F32" s="3" t="inlineStr">
-        <is>
-          <t>?</t>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>Smart-meter and device data</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>Composite performance index (components to check)</t>
+          <t>Peak reduction and system cost targets (DEDALUS aims at 15%)</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>Paper</t>
+          <t>Mixed</t>
         </is>
       </c>
       <c r="I32" s="2" t="n"/>
@@ -2003,50 +2007,186 @@
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
+          <t>Project LEO, Local Energy Oxfordshire (2019 to 2023)</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>SSEN, Oxford, Low Carbon Hub and partners (UK)</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>Resident engagement; trading and market platforms</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>Distribution-grid flexibility market trials, peer-to-peer network capacity trading, local area energy planning</t>
+        </is>
+      </c>
+      <c r="E33" s="3" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>More than 100 monitoring stations</t>
+        </is>
+      </c>
+      <c r="G33" s="3" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="H33" s="2" t="inlineStr">
+        <is>
+          <t>Final report public</t>
+        </is>
+      </c>
+      <c r="I33" s="2" t="inlineStr">
+        <is>
+          <t>https://www.lowcarbonhub.org/wp-content/uploads/2023/02/LEO-Final-Report-Web_lr.pdf</t>
+        </is>
+      </c>
+      <c r="J33" s="2" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>Energy community KPI framework (Giannuzzo et al., Energy Reports 2025)</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>Academic paper (Italy)</t>
+        </is>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>Framework, not software</t>
+        </is>
+      </c>
+      <c r="E34" s="3" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="F34" s="3" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="G34" s="2" t="inlineStr">
+        <is>
+          <t>25 KPIs in four domains: energy, economic, social, environmental; for planning, operation, monitoring and benchmarking</t>
+        </is>
+      </c>
+      <c r="H34" s="2" t="inlineStr">
+        <is>
+          <t>Paper</t>
+        </is>
+      </c>
+      <c r="I34" s="2" t="n"/>
+      <c r="J34" s="2" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>Integrated Energy Community Performance Index (IECPI)</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>Academic proposal</t>
+        </is>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>Composite index, not software</t>
+        </is>
+      </c>
+      <c r="E35" s="3" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="F35" s="3" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="G35" s="2" t="inlineStr">
+        <is>
+          <t>Composite performance index (components to check)</t>
+        </is>
+      </c>
+      <c r="H35" s="2" t="inlineStr">
+        <is>
+          <t>Paper</t>
+        </is>
+      </c>
+      <c r="I35" s="2" t="n"/>
+      <c r="J35" s="2" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
           <t>Smart Energy Communities Benchmark (QUEST and Pollution Probe, 2020)</t>
         </is>
       </c>
-      <c r="B33" s="2" t="inlineStr">
+      <c r="B36" s="2" t="inlineStr">
         <is>
           <t>QUEST Canada and Pollution Probe</t>
         </is>
       </c>
-      <c r="C33" s="2" t="inlineStr">
+      <c r="C36" s="2" t="inlineStr">
         <is>
           <t>Assessment per municipality</t>
         </is>
       </c>
-      <c r="D33" s="2" t="inlineStr">
+      <c r="D36" s="2" t="inlineStr">
         <is>
           <t>Self-assessment against ten indicators</t>
         </is>
       </c>
-      <c r="E33" s="3" t="inlineStr">
-        <is>
-          <t>?</t>
-        </is>
-      </c>
-      <c r="F33" s="2" t="inlineStr">
+      <c r="E36" s="3" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="inlineStr">
         <is>
           <t>Municipal self-reporting; nine pilot communities</t>
         </is>
       </c>
-      <c r="G33" s="2" t="inlineStr">
+      <c r="G36" s="2" t="inlineStr">
         <is>
           <t>Ten indicators: five on capacity (governance, staff, data, financials, strategy), five on outcomes (land use, energy networks, water and waste, transportation, buildings)</t>
         </is>
       </c>
-      <c r="H33" s="2" t="inlineStr">
+      <c r="H36" s="2" t="inlineStr">
         <is>
           <t>Public report</t>
         </is>
       </c>
-      <c r="I33" s="2" t="inlineStr">
+      <c r="I36" s="2" t="inlineStr">
         <is>
           <t>https://questcanada.org/project/is-your-community-energy-smart/</t>
         </is>
       </c>
-      <c r="J33" s="2" t="inlineStr"/>
+      <c r="J36" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>